<commit_message>
Atualização automática - Planilha ReceitaxDespesa
</commit_message>
<xml_diff>
--- a/Grafico_Grupo de Despesa.xlsx
+++ b/Grafico_Grupo de Despesa.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Rei-1cpd003\coord_plan_institucional\DADOS CPI\Orçamento\2026\EXECUÇÃO ORÇAMENTÁRIA\RELEXORC_CSV\Saida_PowerBI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\172.17.1.6\coord_plan_institucional\DADOS CPI\Orçamento\2026\EXECUÇÃO ORÇAMENTÁRIA\RELEXORC_CSV\Saida_PowerBI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8707B50-AA76-4BE6-B411-F71B4AF47C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED73D6C-1DDF-4CA2-A373-22F4D386C175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BD803231-520B-43E5-B415-970328918330}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD803231-520B-43E5-B415-970328918330}"/>
   </bookViews>
   <sheets>
     <sheet name="ReceitaXDespesa" sheetId="3" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2834,7 +2834,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5606F569-D500-4B4F-95B4-2EACD5DAD170}" name="Tabela dinâmica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5606F569-D500-4B4F-95B4-2EACD5DAD170}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A1:C18" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="3">
     <pivotField showAll="0"/>
@@ -3573,7 +3573,10 @@
       <c r="B35" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="1"/>
+      <c r="C35" s="1">
+        <f>87564092.21/1000000</f>
+        <v>87.564092209999998</v>
+      </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="30">
@@ -3582,7 +3585,10 @@
       <c r="B36" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="1"/>
+      <c r="C36" s="1">
+        <f>45147568.89/1000000</f>
+        <v>45.147568890000002</v>
+      </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="30">
@@ -3593,7 +3599,7 @@
       </c>
       <c r="C37" s="1">
         <f>C35-C36</f>
-        <v>0</v>
+        <v>42.416523319999996</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>